<commit_message>
vault backup: 2026-03-11 23:18:57
Affected files:
.obsidian/workspace.json
Work/Research/Research Sources Database.md
Work/Task List/Mech Tasks.md
Work/Task List/Self Task Dump.md
aerospace_intelligence_database_apac_enriched_v2.xlsx
</commit_message>
<xml_diff>
--- a/aerospace_intelligence_database_apac_enriched_v2.xlsx
+++ b/aerospace_intelligence_database_apac_enriched_v2.xlsx
@@ -7,7 +7,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A127CC21-BA47-4788-9150-6B71F4B290E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1056C869-FA27-46F0-9ECB-453EF34DDB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
@@ -26,17 +26,17 @@
     <sheet name="Asian Space Ecosystem" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="true">'Asian Space Ecosystem'!$A$1:$N$100</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Master Database'!$A$1:$N$392</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="true">'Test Facilities'!$A$1:$N$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="true">'CubeSat Components'!$A$1:$N$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="true">'Components'!$A$1:$N$84</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="true">'Propulsion'!$A$1:$N$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="true">'Remote Sensing'!$A$1:$N$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="true">'SSA Tools'!$A$1:$N$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="true">'UAV Aerospace'!$A$1:$N$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="true">'Launch'!$A$1:$N$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="true">'Bus Manufacturers'!$A$1:$N$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="false">'Launch'!$A$1:$N$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="false">'Asian Space Ecosystem'!$A$1:$N$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="false">'Master Database'!$A$1:$N$392</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="false">'Components'!$A$1:$N$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="false">'Bus Manufacturers'!$A$1:$N$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="false">'SSA Tools'!$A$1:$N$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="false">'Propulsion'!$A$1:$N$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="false">'Test Facilities'!$A$1:$N$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="false">'UAV Aerospace'!$A$1:$N$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="false">'CubeSat Components'!$A$1:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="false">'Remote Sensing'!$A$1:$N$54</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -6344,17 +6344,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <sz val="11.00"/>
       <b/>
       <color rgb="FFFFFFFF"/>
       <family val="2"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <name val="Arial"/>
       <sz val="10.00"/>
       <b/>
       <family val="2"/>
-      <name val="Arial"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -6363,24 +6363,24 @@
       <family val="2"/>
     </font>
     <font>
+      <name val="Arial"/>
       <u val="single"/>
       <color rgb="FF0563C1"/>
       <family val="2"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <name val="Arial"/>
       <sz val="10.00"/>
       <i/>
       <color rgb="FF666666"/>
       <family val="2"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <name val="Arial"/>
       <sz val="16.00"/>
       <b/>
       <color rgb="FF000000"/>
       <family val="2"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="8">
@@ -6398,7 +6398,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF17365D"/>
+        <fgColor rgb="FFEEF5FB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6422,7 +6422,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEF5FB"/>
+        <fgColor rgb="FF17365D"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6441,70 +6441,70 @@
     <xf fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" applyFont="1" fillId="4" applyFill="1"/>
-    <xf fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf fontId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="3" applyFont="1"/>
-    <xf fontId="2" applyFont="1" applyAlignment="1">
+    <xf fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="4" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+    <xf fontId="4" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" applyFont="1" fillId="4" applyFill="1"/>
+    <xf fontId="3" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="5" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="4" applyFont="1" applyAlignment="1">
+    <xf fontId="6" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="6" applyFont="1" applyAlignment="1">
+    <xf fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="1" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" applyAlignment="1">
+    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" applyAlignment="1">
+    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="5" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" applyAlignment="1">
+    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf xfId="1" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" applyAlignment="1">
+    <xf xfId="2" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1"/>
-    <xf xfId="2" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1"/>
+    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" applyAlignment="1">
+    <xf xfId="5" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="4" applyFill="1"/>
+    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="4" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="normal" xfId="0" builtinId="0"/>

</xml_diff>